<commit_message>
Adding the material of infomdwr
</commit_message>
<xml_diff>
--- a/Teaching/course_schedule.xlsx
+++ b/Teaching/course_schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hakim/git/infomdwr/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hakim/git/mywebsite/hqahtan.github.io/Teaching/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD5929E8-B246-2648-9BC7-32614649B1BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DD2E581-42AB-174F-9B7F-FA89EFD02F6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1800" yWindow="620" windowWidth="23260" windowHeight="13900" xr2:uid="{72E94DF8-02B7-44D7-9115-6D7B922CAFF9}"/>
+    <workbookView xWindow="1800" yWindow="620" windowWidth="34280" windowHeight="19560" xr2:uid="{72E94DF8-02B7-44D7-9115-6D7B922CAFF9}"/>
   </bookViews>
   <sheets>
     <sheet name="course_schedule_2025" sheetId="1" r:id="rId1"/>
@@ -185,15 +185,6 @@
     <t>Supervised learning: Regression models in R</t>
   </si>
   <si>
-    <t>https://infomdwr.nl/lectures/week_4/3_visualization_1.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_5/1_visualization_2.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_5/2_regression_1_redacted.pdf</t>
-  </si>
-  <si>
     <t>Supervised learning: model evaluation</t>
   </si>
   <si>
@@ -239,51 +230,9 @@
     <t>Algorithmic fairness</t>
   </si>
   <si>
-    <t>https://infomdwr.nl/lectures/week_6/1_regression_2.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_6/2_regression_3.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_6/3_deep_learning.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_7/1_missing_data_1.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_7/2_missing_data_2.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_7/3_clustering_1.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_8/1_clustering_2.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_8/2_text_mining_1.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_8/3_text_mining_2.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_1/1_setup/setup.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/assignments/assignment_1.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_1/2_DataModels.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_1/1_introduction.pdf</t>
-  </si>
-  <si>
     <t>Hetero. data analysis &amp; string similarity</t>
   </si>
   <si>
-    <t>https://infomdwr.nl/assignments/assignment_2.html</t>
-  </si>
-  <si>
     <t>Data visualization</t>
   </si>
   <si>
@@ -296,21 +245,6 @@
     <t>ISLR 5.1, 8.1, 8.2.1, 8.2.2, 8.2.3</t>
   </si>
   <si>
-    <t>https://infomdwr.nl/assignments/assignment_3.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/assignments/assignment_4.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_9/1_TS.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_9/2_DS.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_9/3_Fairness.pdf</t>
-  </si>
-  <si>
     <t>PDA 5, 6.1</t>
   </si>
   <si>
@@ -326,18 +260,6 @@
     <t>Exam Inspection</t>
   </si>
   <si>
-    <t>https://infomdwr.nl/lectures/week_4/1_DP1.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_4/2_DP2.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/exams/FinalExam.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/exams/Mid-TermExam.html</t>
-  </si>
-  <si>
     <t>Functional dependency</t>
   </si>
   <si>
@@ -380,100 +302,178 @@
     <t>Midterm exam (10:00 - 13:00)</t>
   </si>
   <si>
-    <t>https://infomdwr.nl/lectures/week_3/Social.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_2/2_DE_2.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_2/3_ICs.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_3/1_FDs.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_3/2_Indexing_DI.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_3/3_HDA_SS.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/lectures/week_2/1_DE_1.pdf</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_1/2_DataModels/2_DataModels_answers_2738.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_2/1_DE_1/1_DE_1_answers_1063.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_2/2_DE_2/2_DE_2_answers_6271.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_2/3_ICs/3_ICs_answers_3592.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_3/1_FDs/1_FDs_answers_0372.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_3/2_Indexing_DI/2_Indexing_DI_answers_6021.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_3/3_HDA_SS/3_HDA_SS_answers_5529.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_4/1_DP1/1_DP1_answers_8190.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_4/2_DP2/2_DP2_answers_8826.html</t>
-  </si>
-  <si>
     <t>R4DS 1, 3, 9, 10 (optionally 2, 4, 6)</t>
   </si>
   <si>
     <t>R4DS 1, 2, 4, 6</t>
   </si>
   <si>
-    <t>https://infomdwr.nl/labs/week_4/3_data_visualization_1/data_visualization_1_answers.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_5/1_data_visualization_2/data_visualization_2_answers_a20f95b.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_5/2_supervised_1/supervised_1_answers_34b1c2a.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_6/2_supervised_3/supervised_3_answers_3ba2fbb.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_6/3_deep_learning/supervised_4_answers_3gh12s.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_8/1_clustering_2/clustering_2_answers_25ae1b.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_7/1_missing_data_1/missing_data_1_answers_ej4ab45.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_7/2_missing_data_2/missing_data_2_answers_32ksaae.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_7/3_clustering_1/clustering_1_answers_a23b1e3.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_8/2_text_mining_1/text_mining_1_answers_655643.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_8/3_text_mining_2/text_mining_2_answers_3b2f11.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_9/1_TS/1_TS_answers_9022.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_9/2_DS/2_DS_answers_0186.html</t>
-  </si>
-  <si>
-    <t>https://infomdwr.nl/labs/week_9/3_Fairness/3_Fairness_answers_6781.html</t>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_1/1_introduction.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_1/1_setup/setup.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_1/2_DataModels.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_1/2_DataModels/2_DataModels_answers_2738.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_2/1_DE_1.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_2/1_DE_1/1_DE_1_answers_1063.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_2/2_DE_2.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_2/2_DE_2/2_DE_2_answers_6271.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_2/3_ICs.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_2/3_ICs/3_ICs_answers_3592.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_3/1_FDs.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_3/1_FDs/1_FDs_answers_0372.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_3/Social.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_3/2_Indexing_DI.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_3/2_Indexing_DI/2_Indexing_DI_answers_6021.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_3/3_HDA_SS.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_3/3_HDA_SS/3_HDA_SS_answers_5529.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_4/1_DP1.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_4/1_DP1/1_DP1_answers_8190.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/assignments/assignment_1.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_4/2_DP2.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_4/2_DP2/2_DP2_answers_8826.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_4/3_visualization_1.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_4/3_data_visualization_1/data_visualization_1_answers.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_5/1_visualization_2.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_5/1_data_visualization_2/data_visualization_2_answers_a20f95b.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_5/2_regression_1_redacted.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_5/2_supervised_1/supervised_1_answers_34b1c2a.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/exams/Mid-TermExam.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/assignments/assignment_2.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_6/1_regression_2.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/assignments/assignment_3.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_6/2_regression_3.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_6/2_supervised_3/supervised_3_answers_3ba2fbb.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_6/3_deep_learning.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_6/3_deep_learning/supervised_4_answers_3gh12s.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_7/1_missing_data_1.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_7/1_missing_data_1/missing_data_1_answers_ej4ab45.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_7/2_missing_data_2.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_7/2_missing_data_2/missing_data_2_answers_32ksaae.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_7/3_clustering_1.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_7/3_clustering_1/clustering_1_answers_a23b1e3.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_8/1_clustering_2.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_8/1_clustering_2/clustering_2_answers_25ae1b.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_8/2_text_mining_1.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_8/2_text_mining_1/text_mining_1_answers_655643.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_8/3_text_mining_2.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_8/3_text_mining_2/text_mining_2_answers_3b2f11.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_9/1_TS.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_9/1_TS/1_TS_answers_9022.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_9/2_DS.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_9/2_DS/2_DS_answers_0186.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/lectures/week_9/3_Fairness.pdf</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/labs/week_9/3_Fairness/3_Fairness_answers_6781.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/assignments/assignment_4.html</t>
+  </si>
+  <si>
+    <t>https://hqahtan.github.io/Teaching/exams/FinalExam.html</t>
   </si>
 </sst>
 </file>
@@ -911,7 +911,7 @@
         <v>37</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>16</v>
@@ -931,10 +931,10 @@
         <v>38</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>130</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="16" x14ac:dyDescent="0.2">
@@ -951,7 +951,7 @@
         <v>39</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>15</v>
@@ -971,7 +971,7 @@
         <v>39</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>120</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="16" x14ac:dyDescent="0.2">
@@ -988,7 +988,7 @@
         <v>40</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>119</v>
+        <v>93</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>31</v>
@@ -1009,7 +1009,7 @@
         <v>40</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>121</v>
+        <v>94</v>
       </c>
       <c r="I7" s="4"/>
     </row>
@@ -1024,13 +1024,13 @@
         <v>26</v>
       </c>
       <c r="D8" t="s">
-        <v>103</v>
+        <v>77</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="I8" s="4"/>
     </row>
@@ -1045,10 +1045,10 @@
         <v>27</v>
       </c>
       <c r="D9" t="s">
-        <v>103</v>
+        <v>77</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>122</v>
+        <v>96</v>
       </c>
       <c r="I9" s="4"/>
     </row>
@@ -1066,7 +1066,7 @@
         <v>41</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>12</v>
@@ -1087,7 +1087,7 @@
         <v>41</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>123</v>
+        <v>98</v>
       </c>
       <c r="I11" s="4"/>
     </row>
@@ -1102,10 +1102,10 @@
         <v>26</v>
       </c>
       <c r="D12" t="s">
+        <v>73</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>99</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>116</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>14</v>
@@ -1123,10 +1123,10 @@
         <v>27</v>
       </c>
       <c r="D13" t="s">
-        <v>99</v>
+        <v>73</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>124</v>
+        <v>100</v>
       </c>
       <c r="I13" s="4"/>
     </row>
@@ -1138,13 +1138,13 @@
         <v>45916</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>93</v>
+        <v>71</v>
       </c>
       <c r="D14" t="s">
-        <v>102</v>
+        <v>76</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="I14" s="4"/>
     </row>
@@ -1159,13 +1159,13 @@
         <v>26</v>
       </c>
       <c r="D15" t="s">
-        <v>100</v>
+        <v>74</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>101</v>
+        <v>75</v>
       </c>
       <c r="I15" s="4"/>
     </row>
@@ -1180,10 +1180,10 @@
         <v>27</v>
       </c>
       <c r="D16" t="s">
-        <v>100</v>
+        <v>74</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>125</v>
+        <v>103</v>
       </c>
       <c r="I16" s="4"/>
     </row>
@@ -1198,10 +1198,10 @@
         <v>26</v>
       </c>
       <c r="D17" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>13</v>
@@ -1219,10 +1219,10 @@
         <v>27</v>
       </c>
       <c r="D18" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>126</v>
+        <v>105</v>
       </c>
       <c r="I18" s="4"/>
     </row>
@@ -1240,10 +1240,10 @@
         <v>42</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>91</v>
+        <v>69</v>
       </c>
       <c r="I19" s="4"/>
     </row>
@@ -1261,7 +1261,7 @@
         <v>42</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>127</v>
+        <v>107</v>
       </c>
       <c r="I20" s="4"/>
     </row>
@@ -1276,10 +1276,10 @@
         <v>28</v>
       </c>
       <c r="D21" t="s">
-        <v>105</v>
+        <v>79</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>76</v>
+        <v>108</v>
       </c>
       <c r="I21" s="4"/>
     </row>
@@ -1297,10 +1297,10 @@
         <v>43</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>92</v>
+        <v>70</v>
       </c>
       <c r="I22" s="4"/>
     </row>
@@ -1318,7 +1318,7 @@
         <v>43</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="I23" s="4"/>
     </row>
@@ -1333,13 +1333,13 @@
         <v>26</v>
       </c>
       <c r="D24" t="s">
-        <v>81</v>
-      </c>
-      <c r="E24" t="s">
-        <v>48</v>
+        <v>64</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>111</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>129</v>
+        <v>87</v>
       </c>
       <c r="I24" s="4"/>
     </row>
@@ -1354,10 +1354,10 @@
         <v>27</v>
       </c>
       <c r="D25" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>131</v>
+        <v>112</v>
       </c>
       <c r="I25" s="4"/>
     </row>
@@ -1374,11 +1374,11 @@
       <c r="D26" t="s">
         <v>44</v>
       </c>
-      <c r="E26" t="s">
-        <v>49</v>
+      <c r="E26" s="3" t="s">
+        <v>113</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>129</v>
+        <v>87</v>
       </c>
       <c r="I26" s="4"/>
     </row>
@@ -1396,7 +1396,7 @@
         <v>45</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
       <c r="I27" s="4"/>
     </row>
@@ -1413,11 +1413,11 @@
       <c r="D28" t="s">
         <v>46</v>
       </c>
-      <c r="E28" t="s">
-        <v>50</v>
+      <c r="E28" s="3" t="s">
+        <v>115</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="I28" s="4"/>
     </row>
@@ -1435,7 +1435,7 @@
         <v>47</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>133</v>
+        <v>116</v>
       </c>
       <c r="I29" s="4"/>
     </row>
@@ -1482,10 +1482,10 @@
         <v>29</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>112</v>
+        <v>86</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="I32" s="4"/>
     </row>
@@ -1500,10 +1500,10 @@
         <v>28</v>
       </c>
       <c r="D33" t="s">
-        <v>104</v>
+        <v>78</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>80</v>
+        <v>118</v>
       </c>
       <c r="I33" s="4"/>
     </row>
@@ -1518,13 +1518,13 @@
         <v>26</v>
       </c>
       <c r="D34" t="s">
-        <v>51</v>
-      </c>
-      <c r="E34" t="s">
-        <v>66</v>
+        <v>48</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>119</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="I34" s="4"/>
     </row>
@@ -1539,10 +1539,10 @@
         <v>27</v>
       </c>
       <c r="D35" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>85</v>
+        <v>120</v>
       </c>
       <c r="I35" s="4"/>
     </row>
@@ -1557,10 +1557,10 @@
         <v>26</v>
       </c>
       <c r="D36" t="s">
-        <v>52</v>
-      </c>
-      <c r="E36" t="s">
-        <v>67</v>
+        <v>49</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>121</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>19</v>
@@ -1578,10 +1578,10 @@
         <v>27</v>
       </c>
       <c r="D37" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="I37" s="4"/>
     </row>
@@ -1596,10 +1596,10 @@
         <v>26</v>
       </c>
       <c r="D38" t="s">
-        <v>53</v>
-      </c>
-      <c r="E38" t="s">
-        <v>68</v>
+        <v>50</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>123</v>
       </c>
       <c r="F38" s="1" t="s">
         <v>20</v>
@@ -1617,10 +1617,10 @@
         <v>27</v>
       </c>
       <c r="D39" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="I39" s="4"/>
     </row>
@@ -1635,10 +1635,10 @@
         <v>26</v>
       </c>
       <c r="D40" t="s">
-        <v>54</v>
-      </c>
-      <c r="E40" t="s">
-        <v>69</v>
+        <v>51</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>125</v>
       </c>
       <c r="F40" s="1" t="s">
         <v>21</v>
@@ -1656,10 +1656,10 @@
         <v>27</v>
       </c>
       <c r="D41" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="I41" s="4"/>
     </row>
@@ -1674,10 +1674,10 @@
         <v>26</v>
       </c>
       <c r="D42" t="s">
-        <v>56</v>
-      </c>
-      <c r="E42" t="s">
-        <v>70</v>
+        <v>53</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>127</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>21</v>
@@ -1695,10 +1695,10 @@
         <v>27</v>
       </c>
       <c r="D43" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="I43" s="4"/>
     </row>
@@ -1713,10 +1713,10 @@
         <v>26</v>
       </c>
       <c r="D44" t="s">
-        <v>58</v>
-      </c>
-      <c r="E44" t="s">
-        <v>71</v>
+        <v>55</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>129</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>22</v>
@@ -1734,10 +1734,10 @@
         <v>27</v>
       </c>
       <c r="D45" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="I45" s="4"/>
     </row>
@@ -1752,10 +1752,10 @@
         <v>28</v>
       </c>
       <c r="D46" t="s">
-        <v>106</v>
+        <v>80</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>85</v>
+        <v>120</v>
       </c>
       <c r="I46" s="4"/>
     </row>
@@ -1770,10 +1770,10 @@
         <v>26</v>
       </c>
       <c r="D47" t="s">
-        <v>59</v>
-      </c>
-      <c r="E47" t="s">
-        <v>72</v>
+        <v>56</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>131</v>
       </c>
       <c r="F47" s="1" t="s">
         <v>23</v>
@@ -1791,10 +1791,10 @@
         <v>27</v>
       </c>
       <c r="D48" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="I48" s="4"/>
     </row>
@@ -1809,10 +1809,10 @@
         <v>26</v>
       </c>
       <c r="D49" t="s">
-        <v>61</v>
-      </c>
-      <c r="E49" t="s">
-        <v>73</v>
+        <v>58</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>133</v>
       </c>
       <c r="F49" s="1" t="s">
         <v>24</v>
@@ -1830,10 +1830,10 @@
         <v>27</v>
       </c>
       <c r="D50" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="I50" s="4"/>
     </row>
@@ -1845,13 +1845,13 @@
         <v>45953</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>94</v>
+        <v>72</v>
       </c>
       <c r="D51" t="s">
-        <v>108</v>
+        <v>82</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>109</v>
+        <v>83</v>
       </c>
       <c r="I51" s="4"/>
     </row>
@@ -1866,10 +1866,10 @@
         <v>26</v>
       </c>
       <c r="D52" t="s">
-        <v>62</v>
-      </c>
-      <c r="E52" t="s">
-        <v>74</v>
+        <v>59</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>135</v>
       </c>
       <c r="F52" s="1" t="s">
         <v>24</v>
@@ -1887,10 +1887,10 @@
         <v>27</v>
       </c>
       <c r="D53" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="I53" s="4"/>
     </row>
@@ -1905,10 +1905,10 @@
         <v>26</v>
       </c>
       <c r="D54" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>87</v>
+        <v>137</v>
       </c>
       <c r="F54" s="1" t="s">
         <v>17</v>
@@ -1926,10 +1926,10 @@
         <v>27</v>
       </c>
       <c r="D55" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="I55" s="4"/>
     </row>
@@ -1944,10 +1944,10 @@
         <v>26</v>
       </c>
       <c r="D56" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>88</v>
+        <v>139</v>
       </c>
       <c r="F56" s="1" t="s">
         <v>30</v>
@@ -1965,10 +1965,10 @@
         <v>27</v>
       </c>
       <c r="D57" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="I57" s="4"/>
     </row>
@@ -1983,10 +1983,10 @@
         <v>26</v>
       </c>
       <c r="D58" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>89</v>
+        <v>141</v>
       </c>
       <c r="F58" s="1" t="s">
         <v>18</v>
@@ -2004,10 +2004,10 @@
         <v>27</v>
       </c>
       <c r="D59" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="I59" s="4"/>
     </row>
@@ -2022,10 +2022,10 @@
         <v>28</v>
       </c>
       <c r="D60" t="s">
-        <v>107</v>
+        <v>81</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>86</v>
+        <v>143</v>
       </c>
       <c r="I60" s="4"/>
     </row>
@@ -2040,7 +2040,7 @@
         <v>26</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>110</v>
+        <v>84</v>
       </c>
       <c r="E61" s="1"/>
       <c r="I61" s="4"/>
@@ -2072,10 +2072,10 @@
         <v>29</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>111</v>
+        <v>85</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>97</v>
+        <v>144</v>
       </c>
       <c r="I63" s="4"/>
     </row>
@@ -2099,7 +2099,6 @@
       <c r="I65" s="4"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1" xr:uid="{E43B007D-C777-472C-9886-3A0A70544A41}"/>
   <hyperlinks>
     <hyperlink ref="E3" r:id="rId1" xr:uid="{215B70B3-4175-44BC-8514-FB9486B0BCCB}"/>
     <hyperlink ref="E4" r:id="rId2" xr:uid="{1243CD25-F332-4343-8C78-CA5F2BF28841}"/>
@@ -2123,7 +2122,7 @@
     <hyperlink ref="E57" r:id="rId20" xr:uid="{BC1725AA-DC8B-694D-9C7A-D5C521F104AE}"/>
     <hyperlink ref="E55" r:id="rId21" xr:uid="{3A3EEE13-4993-C244-8151-D4BE3335EB7A}"/>
     <hyperlink ref="E59" r:id="rId22" xr:uid="{968EE3E3-DF2A-974C-A35F-963A81B3820E}"/>
-    <hyperlink ref="E21" r:id="rId23" display="https://infomdwr.nl/lectures/week_1/2_DataModels.pdf" xr:uid="{53830B9A-F5DD-9440-8945-7B193F85CD46}"/>
+    <hyperlink ref="E21" r:id="rId23" xr:uid="{53830B9A-F5DD-9440-8945-7B193F85CD46}"/>
     <hyperlink ref="E19" r:id="rId24" xr:uid="{8700939E-E594-6C48-AA4B-95D8E27659DB}"/>
     <hyperlink ref="E22" r:id="rId25" xr:uid="{FECCE109-5902-DE4D-BE91-B9388EAF65BC}"/>
     <hyperlink ref="E20" r:id="rId26" xr:uid="{366EF8F7-2C76-BB4D-B718-50632CFA9D29}"/>
@@ -2144,6 +2143,21 @@
     <hyperlink ref="E14" r:id="rId41" xr:uid="{02A2565C-E883-5C4D-9896-319A3AF5E2DD}"/>
     <hyperlink ref="E27" r:id="rId42" xr:uid="{14708980-9765-4ED2-A658-548340641D11}"/>
     <hyperlink ref="E45" r:id="rId43" xr:uid="{FC400CD8-3E9C-493B-A934-815BF27E4D00}"/>
+    <hyperlink ref="E24" r:id="rId44" xr:uid="{9E4B0502-6DFF-FE48-BD70-318E676BF620}"/>
+    <hyperlink ref="E26" r:id="rId45" xr:uid="{15837120-0D7B-2648-9721-6ED09968605C}"/>
+    <hyperlink ref="E28" r:id="rId46" xr:uid="{BEA2DD69-6892-3B43-B758-FB7202D9CE00}"/>
+    <hyperlink ref="E34" r:id="rId47" xr:uid="{094BDC56-07AA-7842-A15B-CFA790E4D266}"/>
+    <hyperlink ref="E36" r:id="rId48" xr:uid="{9D892C4D-8882-C743-B152-1854EF81D3D3}"/>
+    <hyperlink ref="E38" r:id="rId49" xr:uid="{C5AB0037-F4B7-8D4C-8711-04092E0FE981}"/>
+    <hyperlink ref="E39" r:id="rId50" xr:uid="{4298D4FD-B496-B34A-8BCF-1C18501346D7}"/>
+    <hyperlink ref="E40" r:id="rId51" xr:uid="{8EE0C7DF-2E61-A84D-9FE5-889F977C88FC}"/>
+    <hyperlink ref="E41" r:id="rId52" xr:uid="{41D4C93C-4A9A-E242-B624-7A1CD5EC3D0E}"/>
+    <hyperlink ref="E42" r:id="rId53" xr:uid="{4C8D6ADF-B5CE-8947-95A7-90DD625BFC18}"/>
+    <hyperlink ref="E43" r:id="rId54" xr:uid="{29F4B09B-1437-E54D-9C76-694966E469DE}"/>
+    <hyperlink ref="E44" r:id="rId55" xr:uid="{8F57ED28-3752-4148-A209-149CF341FB52}"/>
+    <hyperlink ref="E47" r:id="rId56" xr:uid="{AFBE6F55-7646-F14F-A1BF-113EC631C71A}"/>
+    <hyperlink ref="E49" r:id="rId57" xr:uid="{92D6274D-1004-904A-9189-178C168688B6}"/>
+    <hyperlink ref="E52" r:id="rId58" xr:uid="{BC8AE8EB-5AA7-B747-AE98-53EEDAB872CD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>